<commit_message>
SkyG Speed 90 C6-9: ready-to-print sliced files with supports (H2S, H2D)
</commit_message>
<xml_diff>
--- a/c6/downloads/C6/SkyG-Speed-90-C6-9-BOM.xlsx
+++ b/c6/downloads/C6/SkyG-Speed-90-C6-9-BOM.xlsx
@@ -3369,10 +3369,10 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>6.2</v>
+        <v>6.6</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>0.65</v>
+        <v>0.75</v>
       </c>
       <c r="E5" s="4" t="n">
         <v>2</v>
@@ -3395,10 +3395,10 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>5.9</v>
+        <v>6.2</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.66</v>
       </c>
       <c r="E6" s="7" t="n">
         <v>2</v>
@@ -3421,10 +3421,10 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>3.9</v>
+        <v>4.1</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>0.39</v>
+        <v>0.49</v>
       </c>
       <c r="E7" s="4" t="n">
         <v>2</v>
@@ -3447,10 +3447,10 @@
         </is>
       </c>
       <c r="C8" s="7" t="n">
-        <v>4.3</v>
+        <v>4.6</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>0.41</v>
+        <v>0.5</v>
       </c>
       <c r="E8" s="7" t="n">
         <v>2</v>
@@ -3473,10 +3473,10 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>0.4</v>
+        <v>0.5</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>0.04</v>
+        <v>0.14</v>
       </c>
       <c r="E9" s="4" t="n">
         <v>2</v>
@@ -3502,7 +3502,7 @@
         <v>0.5</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>0.06</v>
+        <v>0.16</v>
       </c>
       <c r="E10" s="7" t="n">
         <v>2</v>
@@ -3528,7 +3528,7 @@
         <v>0.5</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>0.06</v>
+        <v>0.16</v>
       </c>
       <c r="E11" s="4" t="n">
         <v>2</v>
@@ -3551,10 +3551,10 @@
         </is>
       </c>
       <c r="C12" s="7" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="D12" s="7" t="n">
-        <v>0.06</v>
+        <v>0.16</v>
       </c>
       <c r="E12" s="7" t="n">
         <v>2</v>
@@ -3577,10 +3577,10 @@
         </is>
       </c>
       <c r="C13" s="4" t="n">
-        <v>8.5</v>
+        <v>9.4</v>
       </c>
       <c r="D13" s="4" t="n">
-        <v>0.79</v>
+        <v>0.92</v>
       </c>
       <c r="E13" s="4" t="n">
         <v>2</v>
@@ -3603,10 +3603,10 @@
         </is>
       </c>
       <c r="C14" s="7" t="n">
-        <v>6.7</v>
+        <v>7.4</v>
       </c>
       <c r="D14" s="7" t="n">
-        <v>0.7</v>
+        <v>0.83</v>
       </c>
       <c r="E14" s="7" t="n">
         <v>2</v>
@@ -3632,7 +3632,7 @@
         <v>17.4</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>1.93</v>
+        <v>1.97</v>
       </c>
       <c r="E15" s="4" t="n">
         <v>2</v>
@@ -3655,10 +3655,10 @@
         </is>
       </c>
       <c r="C16" s="7" t="n">
-        <v>21.7</v>
+        <v>22.5</v>
       </c>
       <c r="D16" s="7" t="n">
-        <v>2.18</v>
+        <v>2.23</v>
       </c>
       <c r="E16" s="7" t="n">
         <v>2</v>
@@ -3681,10 +3681,10 @@
         </is>
       </c>
       <c r="C17" s="4" t="n">
-        <v>7.4</v>
+        <v>7.6</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>1.04</v>
+        <v>1.27</v>
       </c>
       <c r="E17" s="4" t="n">
         <v>2</v>
@@ -3710,7 +3710,7 @@
         <v>3.8</v>
       </c>
       <c r="D18" s="7" t="n">
-        <v>0.95</v>
+        <v>1.03</v>
       </c>
       <c r="E18" s="7" t="n">
         <v>2</v>
@@ -3733,10 +3733,10 @@
         </is>
       </c>
       <c r="C19" s="4" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="D19" s="4" t="n">
-        <v>0.21</v>
+        <v>0.3</v>
       </c>
       <c r="E19" s="4" t="n">
         <v>2</v>
@@ -3759,10 +3759,10 @@
         </is>
       </c>
       <c r="C20" s="7" t="n">
-        <v>16.3</v>
+        <v>17.1</v>
       </c>
       <c r="D20" s="7" t="n">
-        <v>2.6</v>
+        <v>2.69</v>
       </c>
       <c r="E20" s="7" t="n">
         <v>1</v>
@@ -3785,10 +3785,10 @@
         </is>
       </c>
       <c r="C21" s="4" t="n">
-        <v>16.3</v>
+        <v>17.1</v>
       </c>
       <c r="D21" s="4" t="n">
-        <v>2.6</v>
+        <v>2.69</v>
       </c>
       <c r="E21" s="4" t="n">
         <v>1</v>
@@ -3811,10 +3811,10 @@
         </is>
       </c>
       <c r="C22" s="7" t="n">
-        <v>2.2</v>
+        <v>2.5</v>
       </c>
       <c r="D22" s="7" t="n">
-        <v>0.5600000000000001</v>
+        <v>0.74</v>
       </c>
       <c r="E22" s="7" t="n">
         <v>1</v>
@@ -3837,10 +3837,10 @@
         </is>
       </c>
       <c r="C23" s="4" t="n">
-        <v>2.3</v>
+        <v>2.4</v>
       </c>
       <c r="D23" s="4" t="n">
-        <v>0.61</v>
+        <v>0.71</v>
       </c>
       <c r="E23" s="4" t="n">
         <v>1</v>
@@ -3863,10 +3863,10 @@
         </is>
       </c>
       <c r="C24" s="7" t="n">
-        <v>3</v>
+        <v>3.2</v>
       </c>
       <c r="D24" s="7" t="n">
-        <v>0.64</v>
+        <v>0.73</v>
       </c>
       <c r="E24" s="7" t="n">
         <v>2</v>
@@ -3889,10 +3889,10 @@
         </is>
       </c>
       <c r="C25" s="4" t="n">
-        <v>2.9</v>
+        <v>3.2</v>
       </c>
       <c r="D25" s="4" t="n">
-        <v>0.63</v>
+        <v>0.73</v>
       </c>
       <c r="E25" s="4" t="n">
         <v>2</v>
@@ -3918,7 +3918,7 @@
         <v>1.9</v>
       </c>
       <c r="D26" s="7" t="n">
-        <v>0.09</v>
+        <v>0.18</v>
       </c>
       <c r="E26" s="7" t="n">
         <v>4</v>
@@ -3941,10 +3941,10 @@
         </is>
       </c>
       <c r="C27" s="4" t="n">
-        <v>4.5</v>
+        <v>4.9</v>
       </c>
       <c r="D27" s="4" t="n">
-        <v>0.9</v>
+        <v>1.02</v>
       </c>
       <c r="E27" s="4" t="n">
         <v>2</v>
@@ -3967,10 +3967,10 @@
         </is>
       </c>
       <c r="C28" s="7" t="n">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="D28" s="7" t="n">
-        <v>0.12</v>
+        <v>0.23</v>
       </c>
       <c r="E28" s="7" t="n">
         <v>4</v>
@@ -3993,10 +3993,10 @@
         </is>
       </c>
       <c r="C29" s="4" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="D29" s="4" t="n">
-        <v>0.03</v>
+        <v>0.12</v>
       </c>
       <c r="E29" s="4" t="n">
         <v>4</v>
@@ -4019,10 +4019,10 @@
         </is>
       </c>
       <c r="C30" s="7" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="D30" s="7" t="n">
-        <v>0.03</v>
+        <v>0.12</v>
       </c>
       <c r="E30" s="7" t="n">
         <v>4</v>
@@ -4045,10 +4045,10 @@
         </is>
       </c>
       <c r="C31" s="4" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="D31" s="4" t="n">
-        <v>0.03</v>
+        <v>0.12</v>
       </c>
       <c r="E31" s="4" t="n">
         <v>4</v>
@@ -4071,10 +4071,10 @@
         </is>
       </c>
       <c r="C32" s="7" t="n">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="D32" s="7" t="n">
-        <v>0.03</v>
+        <v>0.12</v>
       </c>
       <c r="E32" s="7" t="n">
         <v>4</v>
@@ -4088,7 +4088,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>One aircraft (one aircraft with the N0M nose; N0P is an alternative part): 109.5 g, 15.9 h of printing.</t>
+          <t>One aircraft (one aircraft with the N0M nose; N0P is an alternative part): 114.3 g, 17.9 h of printing.</t>
         </is>
       </c>
     </row>

</xml_diff>